<commit_message>
Example output added for README
</commit_message>
<xml_diff>
--- a/Templates/PEATREST_input_scenario_modelling.xlsx
+++ b/Templates/PEATREST_input_scenario_modelling.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://forestresearch-my.sharepoint.com/personal/jacob_osullivan_forestresearch_gov_uk/Documents/Turbines and trees/PEATREST/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="134" documentId="109_{2692C0AF-F37D-4242-A816-1D703B957833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B29538A-C921-460C-9422-7E1FA86E2A71}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="109_{2692C0AF-F37D-4242-A816-1D703B957833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0DE5F39-98BF-4486-84D9-513BF67494E6}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,9 +66,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
+    <customWorkbookView name="Jagadeesh And Dali  - Personal View" guid="{DA59FCE9-3342-40E5-9DAB-341AFC9E9804}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1020" windowHeight="596" activeSheetId="6"/>
+    <customWorkbookView name="soi450 - Personal View" guid="{7ADC3CB4-E91A-4D68-AA62-B94BAF7A6D27}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1020" windowHeight="565" activeSheetId="5"/>
     <customWorkbookView name="soi663 - Personal View" guid="{55FEC4CD-8C58-46CE-8DB2-DCE86527AF45}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1020" windowHeight="596" activeSheetId="5"/>
-    <customWorkbookView name="soi450 - Personal View" guid="{7ADC3CB4-E91A-4D68-AA62-B94BAF7A6D27}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1020" windowHeight="565" activeSheetId="5"/>
-    <customWorkbookView name="Jagadeesh And Dali  - Personal View" guid="{DA59FCE9-3342-40E5-9DAB-341AFC9E9804}" mergeInterval="0" personalView="1" maximized="1" windowWidth="1020" windowHeight="596" activeSheetId="6"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1959,7 +1959,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="280">
+  <cellXfs count="278">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2778,42 +2778,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2859,15 +2823,45 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5925,111 +5919,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>34925</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>330200</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="34" name="Rectangle 135">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000022000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="11325225" y="1416050"/>
-          <a:ext cx="4397375" cy="514350"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="CCFFCC"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="22860" rIns="0" bIns="0" anchor="t" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-GB" sz="800" b="0" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>Note: </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-GB" sz="800" b="0" i="0" u="sng" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>Emissions from felling and timber removal</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-GB" sz="800" b="0" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t>. CARLY REF FOR NEW HARVESTING</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-GB" sz="800" b="0" i="0" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:rPr>
-            <a:t> EMISSIONS FACTOR</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-GB" sz="800" b="0" i="0" strike="noStrike">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-            <a:latin typeface="Arial"/>
-            <a:cs typeface="Arial"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>1095375</xdr:colOff>
       <xdr:row>3</xdr:row>
@@ -8082,7 +7971,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>66</xdr:row>
-          <xdr:rowOff>85725</xdr:rowOff>
+          <xdr:rowOff>82550</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -8140,7 +8029,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>66</xdr:row>
-          <xdr:rowOff>85725</xdr:rowOff>
+          <xdr:rowOff>82550</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -8198,7 +8087,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>101</xdr:row>
-          <xdr:rowOff>104775</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -8256,7 +8145,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>101</xdr:row>
-          <xdr:rowOff>104775</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -8314,7 +8203,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>101</xdr:row>
-          <xdr:rowOff>104775</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -8372,7 +8261,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>101</xdr:row>
-          <xdr:rowOff>104775</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -8430,7 +8319,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>136</xdr:row>
-          <xdr:rowOff>104775</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -8488,7 +8377,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>136</xdr:row>
-          <xdr:rowOff>104775</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -8546,7 +8435,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>136</xdr:row>
-          <xdr:rowOff>104775</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -8604,7 +8493,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>136</xdr:row>
-          <xdr:rowOff>104775</xdr:rowOff>
+          <xdr:rowOff>101600</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -9126,7 +9015,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>67</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -9184,7 +9073,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>67</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -9474,7 +9363,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>103</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -9532,7 +9421,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>103</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -9706,7 +9595,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>138</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -9764,7 +9653,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>138</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -10546,7 +10435,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>71</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -10604,7 +10493,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>71</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -10662,7 +10551,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>71</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -11752,7 +11641,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>52</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -11810,7 +11699,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>52</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -11866,7 +11755,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
-          <xdr:colOff>1095375</xdr:colOff>
+          <xdr:colOff>1092200</xdr:colOff>
           <xdr:row>53</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -11926,7 +11815,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>53</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -11984,7 +11873,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>53</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -12100,7 +11989,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>55</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -12158,7 +12047,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>55</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -12274,7 +12163,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>56</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -12332,7 +12221,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>56</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -12448,7 +12337,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>57</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -12506,7 +12395,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>57</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -12564,7 +12453,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>86</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -12622,7 +12511,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>87</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -12680,7 +12569,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>87</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -13434,7 +13323,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>121</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -13608,7 +13497,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>123</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -13666,7 +13555,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>123</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -13724,7 +13613,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>123</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -13782,7 +13671,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>124</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -13956,7 +13845,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>125</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14014,7 +13903,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>125</xdr:row>
-          <xdr:rowOff>180975</xdr:rowOff>
+          <xdr:rowOff>177800</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14072,7 +13961,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>125</xdr:row>
-          <xdr:rowOff>180975</xdr:rowOff>
+          <xdr:rowOff>177800</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14130,7 +14019,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>126</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14188,7 +14077,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>126</xdr:row>
-          <xdr:rowOff>180975</xdr:rowOff>
+          <xdr:rowOff>177800</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14246,7 +14135,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>126</xdr:row>
-          <xdr:rowOff>180975</xdr:rowOff>
+          <xdr:rowOff>177800</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14362,7 +14251,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>157</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14420,7 +14309,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>157</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14710,7 +14599,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>160</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14768,7 +14657,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>160</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14826,7 +14715,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>160</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14884,7 +14773,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>161</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -14942,7 +14831,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>161</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15000,7 +14889,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>161</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>158750</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15058,7 +14947,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>162</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15116,7 +15005,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>162</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15174,7 +15063,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>192</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15232,7 +15121,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>192</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15290,7 +15179,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>192</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15348,7 +15237,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>193</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15406,7 +15295,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>193</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15464,7 +15353,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>193</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15522,7 +15411,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>195</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15580,7 +15469,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>195</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15638,7 +15527,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>195</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15696,7 +15585,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>196</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15754,7 +15643,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>196</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15812,7 +15701,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>196</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15870,7 +15759,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>197</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15928,7 +15817,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>197</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -15986,7 +15875,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>197</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -16205,7 +16094,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>53</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -16263,7 +16152,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>53</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -16319,7 +16208,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
-          <xdr:colOff>1095375</xdr:colOff>
+          <xdr:colOff>1092200</xdr:colOff>
           <xdr:row>54</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -16379,7 +16268,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>54</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -16437,7 +16326,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>54</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -16843,7 +16732,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>123</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -16901,7 +16790,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>123</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -16959,7 +16848,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>123</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -17017,7 +16906,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>123</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -17075,7 +16964,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>123</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -17133,7 +17022,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>123</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -17191,7 +17080,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>124</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -17597,7 +17486,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>159</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -17655,7 +17544,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>159</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>25400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -17713,7 +17602,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>193</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -17771,7 +17660,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>193</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -17829,7 +17718,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>194</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -17887,7 +17776,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>194</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -17945,7 +17834,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1085850</xdr:colOff>
           <xdr:row>194</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>6350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -19601,25 +19490,25 @@
   <sheetData>
     <row r="1" spans="1:23" ht="13" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="249"/>
-      <c r="C2" s="251" t="s">
+      <c r="B2" s="266"/>
+      <c r="C2" s="268" t="s">
         <v>41</v>
       </c>
-      <c r="D2" s="253" t="s">
+      <c r="D2" s="270" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="254"/>
-      <c r="F2" s="255" t="s">
+      <c r="E2" s="271"/>
+      <c r="F2" s="272" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="256"/>
-      <c r="H2" s="256"/>
-      <c r="I2" s="256"/>
+      <c r="G2" s="273"/>
+      <c r="H2" s="273"/>
+      <c r="I2" s="273"/>
       <c r="J2" s="42"/>
     </row>
     <row r="3" spans="1:23" ht="38" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="250"/>
-      <c r="C3" s="252"/>
+      <c r="B3" s="267"/>
+      <c r="C3" s="269"/>
       <c r="D3" s="32" t="s">
         <v>6</v>
       </c>
@@ -19814,9 +19703,6 @@
       <c r="I12" s="9"/>
       <c r="J12" s="50"/>
       <c r="L12" s="41"/>
-      <c r="T12" s="276"/>
-      <c r="U12" s="276"/>
-      <c r="V12" s="276"/>
     </row>
     <row r="13" spans="1:23" ht="15.5" x14ac:dyDescent="0.25">
       <c r="A13" s="132"/>
@@ -19836,9 +19722,9 @@
       </c>
       <c r="I13" s="9"/>
       <c r="J13" s="50"/>
-      <c r="T13" s="277"/>
-      <c r="U13" s="277"/>
-      <c r="V13" s="277"/>
+      <c r="T13" s="221"/>
+      <c r="U13" s="221"/>
+      <c r="V13" s="221"/>
       <c r="W13" s="221"/>
     </row>
     <row r="14" spans="1:23" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
@@ -19860,9 +19746,9 @@
       <c r="I14" s="9"/>
       <c r="J14" s="50"/>
       <c r="L14" s="41"/>
-      <c r="T14" s="277"/>
-      <c r="U14" s="278"/>
-      <c r="V14" s="277"/>
+      <c r="T14" s="221"/>
+      <c r="U14" s="264"/>
+      <c r="V14" s="221"/>
       <c r="W14" s="221"/>
     </row>
     <row r="15" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -19880,9 +19766,9 @@
       <c r="L15" s="54"/>
       <c r="M15" s="4"/>
       <c r="O15" s="40"/>
-      <c r="T15" s="277"/>
-      <c r="U15" s="279"/>
-      <c r="V15" s="277"/>
+      <c r="T15" s="221"/>
+      <c r="U15" s="265"/>
+      <c r="V15" s="221"/>
       <c r="W15" s="221"/>
     </row>
     <row r="16" spans="1:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -19906,9 +19792,9 @@
       <c r="L16" s="54"/>
       <c r="M16" s="4"/>
       <c r="O16" s="40"/>
-      <c r="T16" s="277"/>
-      <c r="U16" s="279"/>
-      <c r="V16" s="277"/>
+      <c r="T16" s="221"/>
+      <c r="U16" s="265"/>
+      <c r="V16" s="221"/>
       <c r="W16" s="221"/>
     </row>
     <row r="17" spans="2:23" ht="15.5" x14ac:dyDescent="0.2">
@@ -19932,9 +19818,9 @@
       <c r="L17" s="54"/>
       <c r="M17" s="4"/>
       <c r="O17" s="40"/>
-      <c r="T17" s="277"/>
-      <c r="U17" s="279"/>
-      <c r="V17" s="277"/>
+      <c r="T17" s="221"/>
+      <c r="U17" s="265"/>
+      <c r="V17" s="221"/>
       <c r="W17" s="221"/>
     </row>
     <row r="18" spans="2:23" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -19958,9 +19844,9 @@
       <c r="L18" s="54"/>
       <c r="M18" s="4"/>
       <c r="O18" s="40"/>
-      <c r="T18" s="277"/>
-      <c r="U18" s="279"/>
-      <c r="V18" s="277"/>
+      <c r="T18" s="221"/>
+      <c r="U18" s="265"/>
+      <c r="V18" s="221"/>
       <c r="W18" s="221"/>
     </row>
     <row r="19" spans="2:23" ht="13" x14ac:dyDescent="0.2">
@@ -19978,9 +19864,9 @@
       <c r="L19" s="54"/>
       <c r="M19" s="4"/>
       <c r="O19" s="40"/>
-      <c r="T19" s="277"/>
-      <c r="U19" s="279"/>
-      <c r="V19" s="277"/>
+      <c r="T19" s="221"/>
+      <c r="U19" s="265"/>
+      <c r="V19" s="221"/>
       <c r="W19" s="221"/>
     </row>
     <row r="20" spans="2:23" x14ac:dyDescent="0.2">
@@ -20004,9 +19890,9 @@
       <c r="L20" s="54"/>
       <c r="M20" s="4"/>
       <c r="O20" s="40"/>
-      <c r="T20" s="277"/>
-      <c r="U20" s="279"/>
-      <c r="V20" s="277"/>
+      <c r="T20" s="221"/>
+      <c r="U20" s="265"/>
+      <c r="V20" s="221"/>
       <c r="W20" s="221"/>
     </row>
     <row r="21" spans="2:23" ht="15" thickBot="1" x14ac:dyDescent="0.25">
@@ -20030,9 +19916,9 @@
       <c r="L21" s="54"/>
       <c r="M21" s="4"/>
       <c r="O21" s="40"/>
-      <c r="T21" s="277"/>
-      <c r="U21" s="279"/>
-      <c r="V21" s="277"/>
+      <c r="T21" s="221"/>
+      <c r="U21" s="265"/>
+      <c r="V21" s="221"/>
       <c r="W21" s="221"/>
     </row>
     <row r="22" spans="2:23" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -20050,9 +19936,9 @@
       <c r="L22" s="54"/>
       <c r="M22" s="4"/>
       <c r="O22" s="40"/>
-      <c r="T22" s="277"/>
-      <c r="U22" s="279"/>
-      <c r="V22" s="277"/>
+      <c r="T22" s="221"/>
+      <c r="U22" s="265"/>
+      <c r="V22" s="221"/>
       <c r="W22" s="221"/>
     </row>
     <row r="23" spans="2:23" ht="13" x14ac:dyDescent="0.25">
@@ -20067,9 +19953,9 @@
       <c r="H23" s="164"/>
       <c r="I23" s="58"/>
       <c r="J23" s="59"/>
-      <c r="T23" s="277"/>
-      <c r="U23" s="279"/>
-      <c r="V23" s="277"/>
+      <c r="T23" s="221"/>
+      <c r="U23" s="265"/>
+      <c r="V23" s="221"/>
       <c r="W23" s="221"/>
     </row>
     <row r="24" spans="2:23" ht="9" customHeight="1" x14ac:dyDescent="0.2">
@@ -20087,9 +19973,9 @@
       <c r="L24" s="54"/>
       <c r="M24" s="4"/>
       <c r="O24" s="40"/>
-      <c r="T24" s="277"/>
-      <c r="U24" s="279"/>
-      <c r="V24" s="277"/>
+      <c r="T24" s="221"/>
+      <c r="U24" s="265"/>
+      <c r="V24" s="221"/>
       <c r="W24" s="221"/>
     </row>
     <row r="25" spans="2:23" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -20113,9 +19999,6 @@
       <c r="L25" s="39"/>
       <c r="M25" s="4"/>
       <c r="O25" s="40"/>
-      <c r="T25" s="276"/>
-      <c r="U25" s="276"/>
-      <c r="V25" s="276"/>
     </row>
     <row r="26" spans="2:23" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="69"/>
@@ -23968,11 +23851,11 @@
     </row>
     <row r="202" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B202" s="221"/>
-      <c r="C202" s="259"/>
-      <c r="D202" s="259"/>
-      <c r="E202" s="259"/>
-      <c r="F202" s="259"/>
-      <c r="G202" s="259"/>
+      <c r="C202" s="276"/>
+      <c r="D202" s="276"/>
+      <c r="E202" s="276"/>
+      <c r="F202" s="276"/>
+      <c r="G202" s="276"/>
       <c r="H202" s="227"/>
       <c r="I202" s="221"/>
       <c r="J202" s="226"/>
@@ -23980,13 +23863,13 @@
     </row>
     <row r="203" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B203" s="221"/>
-      <c r="C203" s="260"/>
-      <c r="D203" s="260"/>
-      <c r="E203" s="260"/>
-      <c r="F203" s="260"/>
-      <c r="G203" s="260"/>
-      <c r="H203" s="257"/>
-      <c r="I203" s="258"/>
+      <c r="C203" s="277"/>
+      <c r="D203" s="277"/>
+      <c r="E203" s="277"/>
+      <c r="F203" s="277"/>
+      <c r="G203" s="277"/>
+      <c r="H203" s="274"/>
+      <c r="I203" s="275"/>
       <c r="J203" s="221"/>
       <c r="M203" s="4"/>
     </row>
@@ -23997,8 +23880,8 @@
       <c r="E204" s="221"/>
       <c r="F204" s="221"/>
       <c r="G204" s="221"/>
-      <c r="H204" s="257"/>
-      <c r="I204" s="258"/>
+      <c r="H204" s="274"/>
+      <c r="I204" s="275"/>
       <c r="J204" s="221"/>
       <c r="M204" s="4"/>
     </row>
@@ -28343,302 +28226,302 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13" x14ac:dyDescent="0.25">
-      <c r="A1" s="261" t="s">
+      <c r="A1" s="249" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="261" t="s">
+      <c r="B1" s="249" t="s">
         <v>98</v>
       </c>
-      <c r="C1" s="261" t="s">
+      <c r="C1" s="249" t="s">
         <v>99</v>
       </c>
-      <c r="D1" s="261" t="s">
+      <c r="D1" s="249" t="s">
         <v>100</v>
       </c>
-      <c r="E1" s="274" t="s">
+      <c r="E1" s="262" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="13" x14ac:dyDescent="0.25">
-      <c r="A2" s="262" t="s">
+      <c r="A2" s="250" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="262"/>
-      <c r="C2" s="263"/>
-      <c r="D2" s="263"/>
-      <c r="E2" s="264"/>
+      <c r="B2" s="250"/>
+      <c r="C2" s="251"/>
+      <c r="D2" s="251"/>
+      <c r="E2" s="252"/>
     </row>
     <row r="3" spans="1:5" ht="14.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="265" t="s">
+      <c r="A3" s="253" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="265" t="s">
+      <c r="B3" s="253" t="s">
         <v>101</v>
       </c>
-      <c r="C3" s="266">
+      <c r="C3" s="254">
         <v>2880</v>
       </c>
-      <c r="D3" s="266">
+      <c r="D3" s="254">
         <v>2880</v>
       </c>
-      <c r="E3" s="264" t="s">
+      <c r="E3" s="252" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="265" t="s">
+      <c r="A4" s="253" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="265" t="s">
+      <c r="B4" s="253" t="s">
         <v>102</v>
       </c>
-      <c r="C4" s="263">
+      <c r="C4" s="251">
         <v>0.5</v>
       </c>
-      <c r="D4" s="263">
+      <c r="D4" s="251">
         <v>0.5</v>
       </c>
-      <c r="E4" s="267" t="s">
+      <c r="E4" s="255" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="14.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="265" t="s">
+      <c r="A5" s="253" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="265" t="s">
+      <c r="B5" s="253" t="s">
         <v>103</v>
       </c>
-      <c r="C5" s="263">
+      <c r="C5" s="251">
         <v>6</v>
       </c>
-      <c r="D5" s="263">
+      <c r="D5" s="251">
         <v>8</v>
       </c>
-      <c r="E5" s="264" t="s">
+      <c r="E5" s="252" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="265" t="s">
+      <c r="A6" s="253" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="265" t="s">
+      <c r="B6" s="253" t="s">
         <v>104</v>
       </c>
-      <c r="C6" s="263">
+      <c r="C6" s="251">
         <v>4</v>
       </c>
-      <c r="D6" s="263">
+      <c r="D6" s="251">
         <v>7</v>
       </c>
-      <c r="E6" s="264" t="s">
+      <c r="E6" s="252" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="265" t="s">
+      <c r="A7" s="253" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="265" t="s">
+      <c r="B7" s="253" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="263">
+      <c r="C7" s="251">
         <v>1</v>
       </c>
-      <c r="D7" s="263">
+      <c r="D7" s="251">
         <v>1</v>
       </c>
-      <c r="E7" s="264" t="s">
+      <c r="E7" s="252" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="14.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="265" t="s">
+      <c r="A8" s="253" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="265" t="s">
+      <c r="B8" s="253" t="s">
         <v>106</v>
       </c>
-      <c r="C8" s="268">
+      <c r="C8" s="256">
         <v>1.5200000000000001E-3</v>
       </c>
-      <c r="D8" s="268">
+      <c r="D8" s="256">
         <v>1.6559999999999999E-3</v>
       </c>
-      <c r="E8" s="264" t="s">
+      <c r="E8" s="252" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="265" t="s">
+      <c r="A9" s="253" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="265" t="s">
+      <c r="B9" s="253" t="s">
         <v>107</v>
       </c>
-      <c r="C9" s="263">
+      <c r="C9" s="251">
         <v>0.47</v>
       </c>
-      <c r="D9" s="263">
+      <c r="D9" s="251">
         <v>0.47</v>
       </c>
-      <c r="E9" s="267" t="s">
+      <c r="E9" s="255" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="265" t="s">
+      <c r="A10" s="253" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="265" t="s">
+      <c r="B10" s="253" t="s">
         <v>108</v>
       </c>
-      <c r="C10" s="263">
+      <c r="C10" s="251">
         <v>0.25</v>
       </c>
-      <c r="D10" s="263">
+      <c r="D10" s="251">
         <v>0.25</v>
       </c>
-      <c r="E10" s="267" t="s">
+      <c r="E10" s="255" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="265" t="s">
+      <c r="A11" s="253" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="265" t="s">
+      <c r="B11" s="253" t="s">
         <v>109</v>
       </c>
-      <c r="C11" s="269">
+      <c r="C11" s="257">
         <v>1</v>
       </c>
-      <c r="D11" s="269">
+      <c r="D11" s="257">
         <v>1</v>
       </c>
-      <c r="E11" s="267" t="s">
+      <c r="E11" s="255" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="265" t="s">
+      <c r="A12" s="253" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="265" t="s">
+      <c r="B12" s="253" t="s">
         <v>110</v>
       </c>
-      <c r="C12" s="266">
+      <c r="C12" s="254">
         <v>150</v>
       </c>
-      <c r="D12" s="266">
+      <c r="D12" s="254">
         <v>140</v>
       </c>
-      <c r="E12" s="270" t="s">
+      <c r="E12" s="258" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="14.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="265" t="s">
+      <c r="A13" s="253" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="265" t="s">
+      <c r="B13" s="253" t="s">
         <v>111</v>
       </c>
-      <c r="C13" s="263">
+      <c r="C13" s="251">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="D13" s="263">
+      <c r="D13" s="251">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="E13" s="264" t="s">
+      <c r="E13" s="252" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="25" x14ac:dyDescent="0.25">
-      <c r="A14" s="265" t="s">
+      <c r="A14" s="253" t="s">
         <v>112</v>
       </c>
-      <c r="B14" s="265" t="s">
+      <c r="B14" s="253" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="263">
+      <c r="C14" s="251">
         <v>0</v>
       </c>
-      <c r="D14" s="263">
+      <c r="D14" s="251">
         <v>0</v>
       </c>
-      <c r="E14" s="264" t="s">
+      <c r="E14" s="252" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="265" t="s">
+      <c r="A15" s="253" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="265" t="s">
+      <c r="B15" s="253" t="s">
         <v>114</v>
       </c>
-      <c r="C15" s="263">
+      <c r="C15" s="251">
         <v>1</v>
       </c>
-      <c r="D15" s="263">
+      <c r="D15" s="251">
         <v>1</v>
       </c>
-      <c r="E15" s="264" t="s">
+      <c r="E15" s="252" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="265" t="s">
+      <c r="A16" s="253" t="s">
         <v>115</v>
       </c>
-      <c r="B16" s="265" t="s">
+      <c r="B16" s="253" t="s">
         <v>116</v>
       </c>
-      <c r="C16" s="263">
+      <c r="C16" s="251">
         <v>1</v>
       </c>
-      <c r="D16" s="263">
+      <c r="D16" s="251">
         <v>1</v>
       </c>
-      <c r="E16" s="264" t="s">
+      <c r="E16" s="252" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="13" x14ac:dyDescent="0.25">
-      <c r="A17" s="271" t="s">
+      <c r="A17" s="259" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="271"/>
-      <c r="C17" s="272"/>
-      <c r="D17" s="272"/>
-      <c r="E17" s="267"/>
+      <c r="B17" s="259"/>
+      <c r="C17" s="260"/>
+      <c r="D17" s="260"/>
+      <c r="E17" s="255"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="265" t="s">
+      <c r="A18" s="253" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="265" t="s">
+      <c r="B18" s="253" t="s">
         <v>117</v>
       </c>
-      <c r="C18" s="269">
+      <c r="C18" s="257">
         <v>3</v>
       </c>
-      <c r="D18" s="269">
+      <c r="D18" s="257">
         <v>3</v>
       </c>
-      <c r="E18" s="267" t="s">
+      <c r="E18" s="255" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="13" x14ac:dyDescent="0.25">
-      <c r="A19" s="271" t="s">
+      <c r="A19" s="259" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="265" t="s">
+      <c r="A20" s="253" t="s">
         <v>119</v>
       </c>
       <c r="B20" s="219" t="s">
@@ -28667,7 +28550,7 @@
       <c r="D21" s="219">
         <v>0</v>
       </c>
-      <c r="E21" s="264" t="s">
+      <c r="E21" s="252" t="s">
         <v>21</v>
       </c>
     </row>
@@ -28684,12 +28567,12 @@
       <c r="D22" s="219">
         <v>0</v>
       </c>
-      <c r="E22" s="264" t="s">
+      <c r="E22" s="252" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="273" t="s">
+      <c r="A23" s="261" t="s">
         <v>0</v>
       </c>
       <c r="B23" s="219" t="s">
@@ -28701,7 +28584,7 @@
       <c r="D23" s="219">
         <v>0</v>
       </c>
-      <c r="E23" s="264" t="s">
+      <c r="E23" s="252" t="s">
         <v>21</v>
       </c>
     </row>
@@ -28718,7 +28601,7 @@
       <c r="D24" s="219">
         <v>0</v>
       </c>
-      <c r="E24" s="264" t="s">
+      <c r="E24" s="252" t="s">
         <v>21</v>
       </c>
     </row>
@@ -28742,22 +28625,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="13" x14ac:dyDescent="0.3">
-      <c r="A1" s="275" t="s">
+      <c r="A1" s="263" t="s">
         <v>125</v>
       </c>
-      <c r="B1" s="275" t="s">
+      <c r="B1" s="263" t="s">
         <v>126</v>
       </c>
-      <c r="C1" s="275" t="s">
+      <c r="C1" s="263" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="275" t="s">
+      <c r="D1" s="263" t="s">
         <v>128</v>
       </c>
-      <c r="E1" s="275" t="s">
+      <c r="E1" s="263" t="s">
         <v>129</v>
       </c>
-      <c r="F1" s="275" t="s">
+      <c r="F1" s="263" t="s">
         <v>130</v>
       </c>
     </row>
@@ -28965,28 +28848,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="13" x14ac:dyDescent="0.3">
-      <c r="A1" s="275" t="s">
+      <c r="A1" s="263" t="s">
         <v>151</v>
       </c>
-      <c r="B1" s="275" t="s">
+      <c r="B1" s="263" t="s">
         <v>152</v>
       </c>
-      <c r="C1" s="275" t="s">
+      <c r="C1" s="263" t="s">
         <v>161</v>
       </c>
-      <c r="D1" s="275" t="s">
+      <c r="D1" s="263" t="s">
         <v>153</v>
       </c>
-      <c r="E1" s="275" t="s">
+      <c r="E1" s="263" t="s">
         <v>154</v>
       </c>
-      <c r="F1" s="275" t="s">
+      <c r="F1" s="263" t="s">
         <v>155</v>
       </c>
-      <c r="G1" s="275" t="s">
+      <c r="G1" s="263" t="s">
         <v>156</v>
       </c>
-      <c r="H1" s="275" t="s">
+      <c r="H1" s="263" t="s">
         <v>157</v>
       </c>
     </row>

</xml_diff>